<commit_message>
docs(bom): clarify APU=whole-machine ref, add verified ~799$ anchor + price-reliability note
APU row notes the chip isn't sold bare (reference = full Beelink SER8 8845HS ~799$, verified 2026). Analysis block adds the real anchor (a full machine of this tier = 600-800€ -> 300€ even harder) and flags that prices are estimates and some links are whole-machine/category (to confirm via real quotes).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SPARK_BOM.xlsx
+++ b/docs/SPARK_BOM.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Coeur de la console. 8845HS = top 1080p indé mais cher -&gt; tue le 300€. Alternatives moins chères : Z1 non-Extreme, 7640U/8640U, R5 660M.</t>
+          <t>Coeur de la console. 8845HS = top 1080p indé mais cher -&gt; tue le 300€. Alternatives : Z1 non-Extreme, 7640U/8640U, R5 660M. Puce NON vendue nue -&gt; reference achetable = mini-PC complet ~799$ (Beelink SER8, prix verifie 2026).</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
@@ -1244,29 +1244,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="inlineStr">
-        <is>
-          <t>A FAIRE : remplacer mes estimations par de VRAIS devis (APU tray AMD, RAM/SSD volume, devis PCBA, devis moule boitier).</t>
+      <c r="A29" s="17" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>ANCRAGE REEL VERIFIE (2026) : un mini-PC 8845HS COMPLET pret a l'emploi (Beelink SER8) = ~799$ (~740€).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>-&gt; Meme une machine de ce niveau toute faite coute 600-800€. Donc 300€ retail neuf = encore plus dur que l'estime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>FIABILITE PRIX : colonnes = ESTIMATIONS expertes. Certains liens pointent vers une machine entiere ou une categorie, pas la piece exacte -&gt; a confirmer par de vrais devis (APU tray AMD, RAM/SSD volume, devis PCBA JLCPCB/PCBWay, devis moule boitier).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A1:J1"/>
+  <mergeCells count="19">
     <mergeCell ref="A23:J23"/>
+    <mergeCell ref="A32:J32"/>
     <mergeCell ref="A22:J22"/>
     <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A29:J29"/>
+    <mergeCell ref="A20:J20"/>
+    <mergeCell ref="A28:J28"/>
+    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A30:J30"/>
+    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A25:J25"/>
     <mergeCell ref="A18:J18"/>
     <mergeCell ref="A27:J27"/>
     <mergeCell ref="A21:J21"/>
-    <mergeCell ref="A28:J28"/>
-    <mergeCell ref="A29:J29"/>
-    <mergeCell ref="A20:J20"/>
-    <mergeCell ref="A24:J24"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A26:J26"/>
-    <mergeCell ref="A25:J25"/>
-    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A33:J33"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>

</xml_diff>

<commit_message>
docs(bom): add APU 680M vs 780M comparison sheet (price + perf)
Second sheet: 680M (base) vs 780M (Pro) — archi, CU, clocks, relative perf, per-tier game perf (indie/AA/AAA/emulation), upscaling parity, ~40-70 EUR platform price delta, mini-PC proxies. Verdict: 680M enough for indie/creation (cheaper, closer to 300 EUR); 780M = Pro for AA/AAA.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SPARK_BOM.xlsx
+++ b/docs/SPARK_BOM.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM SPARK" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APU 680M vs 780M" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1329,4 +1330,398 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SPARK — APU : Radeon 680M (base) vs 780M (Pro)  ·  prix/perf indicatifs, à valider</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Critère</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Radeon 680M (base)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Radeon 780M (Pro)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Différence / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>RDNA2</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>RDNA3</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>RDNA3 = dual-issue + clocks + IA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Compute Units</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>12 CU</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>12 CU</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Même nombre, mais RDNA3 plus efficace</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Horloge GPU</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>~2.2-2.4 GHz</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>~2.7 GHz</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>780M plus haut</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>APU exemples</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 6800H / 6900HX / 7735HS</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Ryzen 7840HS / 8840HS / 8845HS</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>780M = génération plus récente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Perf GPU relative</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>100 % (base)</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>~+25-30 %</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Écart net sur AA/AAA, faible sur le reste</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Indé / 2D / esport 1080p</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>60 fps facile</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>60 fps facile</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>ÉGAL (les deux suffisent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>AA / un peu vieux 1080p</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>30-45 fps medium</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>45-60 fps medium</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>780M plus confortable</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>AAA récents 1080p</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>720p low + FSR ~30</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>1080p low + FSR 30-45</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>780M = un cran au-dessus</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Émulation GC/Wii/PS2</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
+          <t>OK + marge (réso interne +)</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Les deux bien</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Upscaling FSR / AFMF</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Identique</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Identique</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>PAS lié à la puissance</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>TDP / conso</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>~35-54 W</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>~35-54 W</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Similaire (wall-powered)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Prix plateforme (BOM, volume est.)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>~90-130 €</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>~150-200 €</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Δ ~ +40-70 € pour le 780M</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Mini-PC proxy (retail)</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>~300-400 € (Beelink SER6…)</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>~500-800 € (Beelink SER8…)</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Machine entière, pas la puce seule</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>VERDICT :</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>- Pour de l'INDÉ / esport / rétro / création (FORGE) : 680M = SUFFISANT → choisis-le (moins cher, ~-40-70 € BOM, plus près de 300 €).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>- Pour viser AA/AAA confortables : 780M (= SKU 'Pro', prix plus haut).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>- L'upscaling (FSR/AFMF) est IDENTIQUE sur les deux → le 680M en profite autant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>- Δ prix puce ~40-70 € en volume ; les écarts mini-PC (300 vs 800 €) = machines entières, pas la puce.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>- Stratégie SPARK : 680M = base abordable, 780M = Pro optionnel. (Premium AAA = Strix Halo, autre gamme.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Prix = ESTIMATIONS à confirmer par devis (AMD tray / fabricant).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A19:D19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(bom): add full-machine cost sheet (680M build vs 780M build + retail est.)
Third sheet: same components, only APU differs (680M ~110 vs 780M ~170). TOTAL BOM ~287 vs ~347 EUR; retail x1.5-x1.8 = ~430-516 (680M) vs ~520-625 (780M). Note: 300 EUR retail not reached even with 680M.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SPARK_BOM.xlsx
+++ b/docs/SPARK_BOM.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM SPARK" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="APU 680M vs 780M" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coût machine 680M vs 780M" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0 €"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +68,11 @@
     <font>
       <color rgb="00333333"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -123,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -168,6 +174,15 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1724,4 +1739,334 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SPARK — Coût machine complète : build 680M vs build 780M  ·  prix pro/volume estimés (€)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Composant</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Build 680M (€)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Build 780M (€)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>APU</t>
+        </is>
+      </c>
+      <c r="B3" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="C3" s="10" t="n">
+        <v>170</v>
+      </c>
+      <c r="D3" s="18" t="inlineStr">
+        <is>
+          <t>Seule vraie différence (680M vs 780M, volume)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>RAM 16 Go DDR5 dual-channel</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="D4" s="19" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Stockage NVMe 512 Go</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="D5" s="18" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Carte mère custom (PCBA)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>hors NRE étude</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Refroidissement</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" s="18" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Alimentation</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="D8" s="19" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Boîtier</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D9" s="18" t="inlineStr">
+        <is>
+          <t>hors NRE moule</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Lecteur micro-SD</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D10" s="19" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Manette</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D11" s="18" t="inlineStr">
+        <is>
+          <t>option : vendre à part</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Connecteurs / divers</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" s="19" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Assemblage + test</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="D13" s="18" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL BOM (pièces)</t>
+        </is>
+      </c>
+      <c r="B14" s="15">
+        <f>SUM(B3:B13)</f>
+        <v/>
+      </c>
+      <c r="C14" s="15">
+        <f>SUM(C3:C13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="20" t="inlineStr">
+        <is>
+          <t>hors transport/marge/R&amp;D/marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Prix retail estimé ×1.5 (direct, marge fine)</t>
+        </is>
+      </c>
+      <c r="B15" s="22">
+        <f>B14*1.5</f>
+        <v/>
+      </c>
+      <c r="C15" s="22">
+        <f>C14*1.5</f>
+        <v/>
+      </c>
+      <c r="D15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Prix retail estimé ×1.8 (marge + distrib)</t>
+        </is>
+      </c>
+      <c r="B16" s="22">
+        <f>B14*1.8</f>
+        <v/>
+      </c>
+      <c r="C16" s="22">
+        <f>C14*1.8</f>
+        <v/>
+      </c>
+      <c r="D16" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>LECTURE :</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>- Seule différence = l'APU (680M ~110€ vs 780M ~170€) -&gt; Δ BOM ~ +60€ pour le 780M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>- TOTAL BOM ~ 287€ (680M) vs ~347€ (780M). Retail réaliste = BOM ×1.5 à ×1.8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>- 680M : retail ~430-516€. 780M : retail ~520-625€.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>- =&gt; Le 300€ retail N'EST PAS atteint, même en 680M (BOM déjà ~287€). Pour 300€ : APU encore plus faible (Vega/660M), couper RAM/manette, ou vendre à perte + abo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>- Manette vendue à part = -14€ BOM. APU plus faible = la plus grosse économie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>Prix = ESTIMATIONS (à confirmer par devis AMD tray / fabricant / PCBA / moule).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A19:D19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>